<commit_message>
finale lijst vóór heroriëntering
#72
</commit_message>
<xml_diff>
--- a/prius2/input/lijst-5_v25-08-19.xlsx
+++ b/prius2/input/lijst-5_v25-08-19.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bram_dhondt\Documents\GitHub\prius\prius2\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8E3D13B-F64B-419F-8214-4D26256C15B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5454016-EBAF-4E2B-BF34-9C243AEAED34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{AA2552F2-2547-4780-972A-FBD54CB263EB}"/>
+    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15840" xr2:uid="{AA2552F2-2547-4780-972A-FBD54CB263EB}"/>
   </bookViews>
   <sheets>
     <sheet name="Blad1" sheetId="1" r:id="rId1"/>
@@ -259,11 +259,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standaard" xfId="0" builtinId="0"/>
@@ -602,7 +600,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="29.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="62.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="62.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="4.21875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="27" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.77734375" bestFit="1" customWidth="1"/>
@@ -615,7 +613,7 @@
       <c r="B1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>25</v>
       </c>
       <c r="D1" s="1" t="s">
@@ -635,7 +633,7 @@
       <c r="B2" t="s">
         <v>56</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" t="s">
         <v>0</v>
       </c>
       <c r="D2">
@@ -655,7 +653,7 @@
       <c r="B3" t="s">
         <v>41</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" t="s">
         <v>1</v>
       </c>
       <c r="D3">
@@ -675,7 +673,7 @@
       <c r="B4" t="s">
         <v>31</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" t="s">
         <v>2</v>
       </c>
       <c r="D4">
@@ -695,7 +693,7 @@
       <c r="B5" t="s">
         <v>42</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" t="s">
         <v>3</v>
       </c>
       <c r="D5">
@@ -715,7 +713,7 @@
       <c r="B6" t="s">
         <v>32</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" t="s">
         <v>4</v>
       </c>
       <c r="D6">
@@ -735,7 +733,7 @@
       <c r="B7" t="s">
         <v>50</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" t="s">
         <v>5</v>
       </c>
       <c r="D7">
@@ -755,7 +753,7 @@
       <c r="B8" t="s">
         <v>33</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" t="s">
         <v>6</v>
       </c>
       <c r="D8">
@@ -775,7 +773,7 @@
       <c r="B9" t="s">
         <v>43</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" t="s">
         <v>7</v>
       </c>
       <c r="D9">
@@ -795,7 +793,7 @@
       <c r="B10" t="s">
         <v>44</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" t="s">
         <v>8</v>
       </c>
       <c r="D10">
@@ -815,7 +813,7 @@
       <c r="B11" t="s">
         <v>45</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" t="s">
         <v>9</v>
       </c>
       <c r="D11">
@@ -835,7 +833,7 @@
       <c r="B12" t="s">
         <v>51</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" t="s">
         <v>10</v>
       </c>
       <c r="D12">
@@ -855,7 +853,7 @@
       <c r="B13" t="s">
         <v>37</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" t="s">
         <v>11</v>
       </c>
       <c r="D13">
@@ -875,7 +873,7 @@
       <c r="B14" t="s">
         <v>46</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" t="s">
         <v>12</v>
       </c>
       <c r="D14">
@@ -895,7 +893,7 @@
       <c r="B15" t="s">
         <v>47</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C15" t="s">
         <v>13</v>
       </c>
       <c r="D15">
@@ -915,7 +913,7 @@
       <c r="B16" t="s">
         <v>59</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" t="s">
         <v>14</v>
       </c>
       <c r="D16">
@@ -935,7 +933,7 @@
       <c r="B17" t="s">
         <v>58</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="C17" t="s">
         <v>15</v>
       </c>
       <c r="D17">
@@ -945,7 +943,7 @@
         <v>5</v>
       </c>
       <c r="F17">
-        <v>2367911</v>
+        <v>2367913</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
@@ -955,7 +953,7 @@
       <c r="B18" t="s">
         <v>34</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="C18" t="s">
         <v>16</v>
       </c>
       <c r="D18">
@@ -975,7 +973,7 @@
       <c r="B19" t="s">
         <v>38</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="C19" t="s">
         <v>17</v>
       </c>
       <c r="D19">
@@ -995,7 +993,7 @@
       <c r="B20" t="s">
         <v>35</v>
       </c>
-      <c r="C20" s="3" t="s">
+      <c r="C20" t="s">
         <v>18</v>
       </c>
       <c r="D20">
@@ -1015,7 +1013,7 @@
       <c r="B21" t="s">
         <v>48</v>
       </c>
-      <c r="C21" s="3" t="s">
+      <c r="C21" t="s">
         <v>19</v>
       </c>
       <c r="D21">
@@ -1035,7 +1033,7 @@
       <c r="B22" t="s">
         <v>36</v>
       </c>
-      <c r="C22" s="3" t="s">
+      <c r="C22" t="s">
         <v>20</v>
       </c>
       <c r="D22">
@@ -1055,7 +1053,7 @@
       <c r="B23" t="s">
         <v>49</v>
       </c>
-      <c r="C23" s="3" t="s">
+      <c r="C23" t="s">
         <v>21</v>
       </c>
       <c r="D23">
@@ -1075,7 +1073,7 @@
       <c r="B24" t="s">
         <v>52</v>
       </c>
-      <c r="C24" s="3" t="s">
+      <c r="C24" t="s">
         <v>24</v>
       </c>
       <c r="D24">
@@ -1095,7 +1093,7 @@
       <c r="B25" t="s">
         <v>53</v>
       </c>
-      <c r="C25" s="3" t="s">
+      <c r="C25" t="s">
         <v>22</v>
       </c>
       <c r="D25">
@@ -1115,7 +1113,7 @@
       <c r="B26" t="s">
         <v>54</v>
       </c>
-      <c r="C26" s="3" t="s">
+      <c r="C26" t="s">
         <v>23</v>
       </c>
       <c r="D26">
@@ -1135,7 +1133,7 @@
       <c r="B27" t="s">
         <v>40</v>
       </c>
-      <c r="C27" s="3" t="s">
+      <c r="C27" t="s">
         <v>39</v>
       </c>
       <c r="D27">

</xml_diff>